<commit_message>
final touches on project params, re-ran outputjob
</commit_message>
<xml_diff>
--- a/Project Outputs for UZ_D_Incr_Encoder/04/BOM/BOM_JLC-UZ_D_Incr_Encoder(Default).xlsx
+++ b/Project Outputs for UZ_D_Incr_Encoder/04/BOM/BOM_JLC-UZ_D_Incr_Encoder(Default).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
-  <workbookPr defaultThemeVersion="166925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gauppto\Documents\uz_d_incr_encoder\Project Outputs for UZ_D_Incr_Encoder\04\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIT\UltraZohm\pcb_design\uz_d_incr_encoder\Project Outputs for UZ_D_Incr_Encoder\04\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8CDFF967-5799-4EC2-9556-47A89B3D6419}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{FC5FFB8F-4F61-42E2-813C-B3C9BB727369}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20025" yWindow="3090" windowWidth="16245" windowHeight="16320" xr2:uid="{C462FF56-6152-493A-B57B-719B500BB009}"/>
+    <workbookView xWindow="28680" yWindow="-12300" windowWidth="51840" windowHeight="21120" xr2:uid="{8D24C45B-7569-4115-BF4E-F8F10E910FE7}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM_JLC-UZ_D_Incr_Encoder(Defau" sheetId="1" r:id="rId1"/>
@@ -30,10 +30,12 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
+      <xlwcv:version setVersion="2"/>
     </ext>
   </extLst>
 </workbook>
@@ -45,7 +47,7 @@
     <t>Quantity</t>
   </si>
   <si>
-    <t>Comment</t>
+    <t>Name</t>
   </si>
   <si>
     <t>Designator</t>
@@ -452,7 +454,7 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -532,39 +534,39 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="44546A"/>
+        <a:srgbClr val="0E2841"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E7E6E6"/>
+        <a:srgbClr val="E8E8E8"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4472C4"/>
+        <a:srgbClr val="156082"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="ED7D31"/>
+        <a:srgbClr val="E97132"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="A5A5A5"/>
+        <a:srgbClr val="196B24"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="FFC000"/>
+        <a:srgbClr val="0F9ED5"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="5B9BD5"/>
+        <a:srgbClr val="A02B93"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="70AD47"/>
+        <a:srgbClr val="4EA72E"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0563C1"/>
+        <a:srgbClr val="467886"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="954F72"/>
+        <a:srgbClr val="96607D"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -616,7 +618,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -727,13 +729,6 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
         <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
@@ -742,6 +737,13 @@
           <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -806,34 +808,54 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
+  <a:objectDefaults>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C517E603-C730-4191-B07E-F91F2DAE8609}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EDE640FB-7B55-4675-9DF9-2EF32DA53586}">
   <dimension ref="A1:K23"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="9.7109375" customWidth="1"/>
-    <col min="2" max="2" width="19.28515625" customWidth="1"/>
-    <col min="3" max="3" width="17.85546875" customWidth="1"/>
-    <col min="4" max="4" width="16.7109375" customWidth="1"/>
-    <col min="5" max="5" width="17.140625" customWidth="1"/>
-    <col min="6" max="6" width="16.5703125" customWidth="1"/>
-    <col min="7" max="7" width="24.7109375" customWidth="1"/>
-    <col min="8" max="8" width="8.85546875" customWidth="1"/>
-    <col min="9" max="9" width="10.140625" customWidth="1"/>
-    <col min="10" max="11" width="16.7109375" customWidth="1"/>
+    <col min="1" max="1" width="9.26953125" customWidth="1"/>
+    <col min="2" max="2" width="18.54296875" customWidth="1"/>
+    <col min="3" max="3" width="17.08984375" customWidth="1"/>
+    <col min="4" max="4" width="16" customWidth="1"/>
+    <col min="5" max="5" width="16.36328125" customWidth="1"/>
+    <col min="6" max="6" width="15.90625" customWidth="1"/>
+    <col min="7" max="7" width="23.54296875" customWidth="1"/>
+    <col min="8" max="8" width="8.453125" customWidth="1"/>
+    <col min="9" max="9" width="9.7265625" customWidth="1"/>
+    <col min="10" max="11" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -868,7 +890,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" s="1">
         <v>12</v>
       </c>
@@ -899,7 +921,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3" s="1">
         <v>9</v>
       </c>
@@ -930,7 +952,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" s="1">
         <v>4</v>
       </c>
@@ -961,7 +983,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5" s="1">
         <v>1</v>
       </c>
@@ -992,7 +1014,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A6" s="1">
         <v>3</v>
       </c>
@@ -1021,7 +1043,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A7" s="1">
         <v>2</v>
       </c>
@@ -1052,7 +1074,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A8" s="1">
         <v>3</v>
       </c>
@@ -1085,7 +1107,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9" s="1">
         <v>3</v>
       </c>
@@ -1114,7 +1136,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -1145,7 +1167,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A11" s="1">
         <v>24</v>
       </c>
@@ -1176,7 +1198,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A12" s="1">
         <v>3</v>
       </c>
@@ -1207,7 +1229,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A13" s="1">
         <v>3</v>
       </c>
@@ -1238,7 +1260,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A14" s="1">
         <v>2</v>
       </c>
@@ -1269,7 +1291,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A15" s="1">
         <v>6</v>
       </c>
@@ -1300,7 +1322,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A16" s="1">
         <v>3</v>
       </c>
@@ -1329,7 +1351,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A17" s="1">
         <v>3</v>
       </c>
@@ -1358,7 +1380,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A18" s="1">
         <v>3</v>
       </c>
@@ -1389,7 +1411,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A19" s="1">
         <v>1</v>
       </c>
@@ -1420,7 +1442,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A20" s="1">
         <v>1</v>
       </c>
@@ -1451,7 +1473,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A21" s="1">
         <v>2</v>
       </c>
@@ -1480,7 +1502,7 @@
       </c>
       <c r="K21" s="1"/>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A22" s="1">
         <v>1</v>
       </c>
@@ -1507,7 +1529,7 @@
       </c>
       <c r="K22" s="1"/>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A23" s="1">
         <v>3</v>
       </c>

</xml_diff>

<commit_message>
Wire Connection ergänzt, hat gefehlt! Output job erstellt
</commit_message>
<xml_diff>
--- a/Project Outputs for UZ_D_Incr_Encoder/04/BOM/BOM_JLC-UZ_D_Incr_Encoder(Default).xlsx
+++ b/Project Outputs for UZ_D_Incr_Encoder/04/BOM/BOM_JLC-UZ_D_Incr_Encoder(Default).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIT\UltraZohm\pcb_design\uz_d_incr_encoder\Project Outputs for UZ_D_Incr_Encoder\04\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gauppto\Documents\uz_d_incr_encoder\Project Outputs for UZ_D_Incr_Encoder\04\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FC5FFB8F-4F61-42E2-813C-B3C9BB727369}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{AC57502A-2C62-4E9C-AC0A-BDCF8558465C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-12300" windowWidth="51840" windowHeight="21120" xr2:uid="{8D24C45B-7569-4115-BF4E-F8F10E910FE7}"/>
+    <workbookView xWindow="20025" yWindow="3090" windowWidth="16245" windowHeight="16320" xr2:uid="{13D917C7-0D54-4E7F-8296-7102CDE022AB}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM_JLC-UZ_D_Incr_Encoder(Defau" sheetId="1" r:id="rId1"/>
@@ -30,12 +30,10 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="2"/>
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -47,7 +45,7 @@
     <t>Quantity</t>
   </si>
   <si>
-    <t>Name</t>
+    <t>Comment</t>
   </si>
   <si>
     <t>Designator</t>
@@ -454,7 +452,7 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -534,39 +532,39 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="0E2841"/>
+        <a:srgbClr val="44546A"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E8E8E8"/>
+        <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="156082"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="E97132"/>
+        <a:srgbClr val="ED7D31"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="196B24"/>
+        <a:srgbClr val="A5A5A5"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="0F9ED5"/>
+        <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="A02B93"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="4EA72E"/>
+        <a:srgbClr val="70AD47"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="467886"/>
+        <a:srgbClr val="0563C1"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="96607D"/>
+        <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -618,7 +616,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -729,6 +727,13 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
         <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
@@ -737,13 +742,6 @@
           <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -808,54 +806,34 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
+  <a:objectDefaults/>
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EDE640FB-7B55-4675-9DF9-2EF32DA53586}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{178F88F1-8D6E-4E1C-A2A3-ABAD09FEFEE1}">
   <dimension ref="A1:K23"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.26953125" customWidth="1"/>
-    <col min="2" max="2" width="18.54296875" customWidth="1"/>
-    <col min="3" max="3" width="17.08984375" customWidth="1"/>
-    <col min="4" max="4" width="16" customWidth="1"/>
-    <col min="5" max="5" width="16.36328125" customWidth="1"/>
-    <col min="6" max="6" width="15.90625" customWidth="1"/>
-    <col min="7" max="7" width="23.54296875" customWidth="1"/>
-    <col min="8" max="8" width="8.453125" customWidth="1"/>
-    <col min="9" max="9" width="9.7265625" customWidth="1"/>
-    <col min="10" max="11" width="16" customWidth="1"/>
+    <col min="1" max="1" width="9.7109375" customWidth="1"/>
+    <col min="2" max="2" width="19.28515625" customWidth="1"/>
+    <col min="3" max="3" width="17.85546875" customWidth="1"/>
+    <col min="4" max="4" width="16.7109375" customWidth="1"/>
+    <col min="5" max="5" width="17.140625" customWidth="1"/>
+    <col min="6" max="6" width="16.5703125" customWidth="1"/>
+    <col min="7" max="7" width="24.7109375" customWidth="1"/>
+    <col min="8" max="8" width="8.85546875" customWidth="1"/>
+    <col min="9" max="9" width="10.140625" customWidth="1"/>
+    <col min="10" max="11" width="16.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -890,7 +868,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>12</v>
       </c>
@@ -921,7 +899,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>9</v>
       </c>
@@ -952,7 +930,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>4</v>
       </c>
@@ -983,7 +961,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>1</v>
       </c>
@@ -1014,7 +992,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>3</v>
       </c>
@@ -1043,7 +1021,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>2</v>
       </c>
@@ -1074,7 +1052,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>3</v>
       </c>
@@ -1107,7 +1085,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>3</v>
       </c>
@@ -1136,7 +1114,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -1167,7 +1145,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>24</v>
       </c>
@@ -1198,7 +1176,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>3</v>
       </c>
@@ -1229,7 +1207,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>3</v>
       </c>
@@ -1260,7 +1238,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>2</v>
       </c>
@@ -1291,7 +1269,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>6</v>
       </c>
@@ -1322,7 +1300,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>3</v>
       </c>
@@ -1351,7 +1329,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>3</v>
       </c>
@@ -1380,7 +1358,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>3</v>
       </c>
@@ -1411,7 +1389,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
         <v>1</v>
       </c>
@@ -1442,7 +1420,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
         <v>1</v>
       </c>
@@ -1473,7 +1451,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
         <v>2</v>
       </c>
@@ -1502,7 +1480,7 @@
       </c>
       <c r="K21" s="1"/>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
         <v>1</v>
       </c>
@@ -1529,7 +1507,7 @@
       </c>
       <c r="K22" s="1"/>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
         <v>3</v>
       </c>

</xml_diff>

<commit_message>
fixed outline, fixed X1 position, X2/X3, X4 and X5_i are set to DNP in Default Variant
</commit_message>
<xml_diff>
--- a/Project Outputs for UZ_D_Incr_Encoder/04/BOM/BOM_JLC-UZ_D_Incr_Encoder(Default).xlsx
+++ b/Project Outputs for UZ_D_Incr_Encoder/04/BOM/BOM_JLC-UZ_D_Incr_Encoder(Default).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gauppto\Documents\uz_d_incr_encoder\Project Outputs for UZ_D_Incr_Encoder\04\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AC57502A-2C62-4E9C-AC0A-BDCF8558465C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F77FFD29-53A9-4E5E-9D04-6ADE2E2E6682}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20025" yWindow="3090" windowWidth="16245" windowHeight="16320" xr2:uid="{13D917C7-0D54-4E7F-8296-7102CDE022AB}"/>
+    <workbookView xWindow="20025" yWindow="3090" windowWidth="16245" windowHeight="16320" xr2:uid="{B88F2F2C-2FF7-4C80-8AE6-0E8974D1942D}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM_JLC-UZ_D_Incr_Encoder(Defau" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="120">
   <si>
     <t>Quantity</t>
   </si>
@@ -400,48 +400,6 @@
   </si>
   <si>
     <t>C81457</t>
-  </si>
-  <si>
-    <t>Pin Header</t>
-  </si>
-  <si>
-    <t>X2, X3</t>
-  </si>
-  <si>
-    <t>SAMTEC</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>THROUGH-HOLE .025" SQ POST HEADER</t>
-  </si>
-  <si>
-    <t>SAMTEC_TSW-110-07-F-T</t>
-  </si>
-  <si>
-    <t>TSW-110-07-F-T</t>
-  </si>
-  <si>
-    <t>X4</t>
-  </si>
-  <si>
-    <t>SAMTEC_TSW-106-07-F-D</t>
-  </si>
-  <si>
-    <t>TSW-106-07-F-D</t>
-  </si>
-  <si>
-    <t>X5_1, X5_2, X5_3</t>
-  </si>
-  <si>
-    <t>8 Pin</t>
-  </si>
-  <si>
-    <t>HDR1X8</t>
-  </si>
-  <si>
-    <t>103741-8</t>
   </si>
 </sst>
 </file>
@@ -817,8 +775,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{178F88F1-8D6E-4E1C-A2A3-ABAD09FEFEE1}">
-  <dimension ref="A1:K23"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7531410B-3C9D-4E70-8473-74A988E0CE4E}">
+  <dimension ref="A1:K20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.7109375" customWidth="1"/>
@@ -1451,89 +1409,6 @@
         <v>119</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A21" s="1">
-        <v>2</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="E21" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="F21" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="G21" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="H21" s="1"/>
-      <c r="I21" s="1"/>
-      <c r="J21" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="K21" s="1"/>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A22" s="1">
-        <v>1</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>127</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="E22" s="1"/>
-      <c r="F22" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="G22" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="H22" s="1"/>
-      <c r="I22" s="1"/>
-      <c r="J22" s="2" t="s">
-        <v>129</v>
-      </c>
-      <c r="K22" s="1"/>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A23" s="1">
-        <v>3</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>130</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="E23" s="1"/>
-      <c r="F23" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="G23" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="H23" s="1"/>
-      <c r="I23" s="1"/>
-      <c r="J23" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="K23" s="1"/>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>